<commit_message>
Update Physical Arcitecture Systems - Space Oddity.xlsx
</commit_message>
<xml_diff>
--- a/Space Oddity/Physical Arcitecture Systems - Space Oddity.xlsx
+++ b/Space Oddity/Physical Arcitecture Systems - Space Oddity.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c1c088fba97fd989/Pictures/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4d14bd4a04985854/Documents/GitHub/AIAA-Systems-Engineering-Workshop/Space Oddity/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{F1A67CE8-83FE-40DF-A4B6-0CE8344C5257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{40DB0116-7804-4C28-AB7A-066080E402DC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{40DB0116-7804-4C28-AB7A-066080E402DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -498,12 +498,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE65C89A-5308-4B94-BCA6-975CA2427D55}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="8.88671875" customWidth="1"/>
+    <col min="1" max="2" width="8.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -511,7 +511,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -519,7 +519,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -527,7 +527,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1.1000000000000001</v>
       </c>
@@ -535,7 +535,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -543,7 +543,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -551,7 +551,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -559,7 +559,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1.2</v>
       </c>
@@ -567,7 +567,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -575,7 +575,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -583,7 +583,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1.3</v>
       </c>
@@ -591,7 +591,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -599,7 +599,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -607,7 +607,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -615,7 +615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1.4</v>
       </c>
@@ -623,7 +623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1.5</v>
       </c>
@@ -631,7 +631,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2</v>
       </c>
@@ -639,7 +639,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2.1</v>
       </c>
@@ -647,7 +647,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2.2000000000000002</v>
       </c>
@@ -655,7 +655,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>9</v>
       </c>

</xml_diff>